<commit_message>
Filter by level scenario added
</commit_message>
<xml_diff>
--- a/src/test/testData/FilterLevels.xlsx
+++ b/src/test/testData/FilterLevels.xlsx
@@ -6,7 +6,7 @@
     <workbookView tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" name="Sheet1" sheetId="1"/>
+    <sheet r:id="rId1" name="Levels" sheetId="1"/>
   </sheets>
   <calcPr calcId="0" iterate="1" iterateCount="1000" iterateDelta="0.01"/>
 </workbook>
@@ -34,14 +34,42 @@
 </metadata>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Expert</t>
+  </si>
+  <si>
+    <t>Beginner</t>
+  </si>
+  <si>
+    <t>Intermediate</t>
+  </si>
+  <si>
+    <t>Advanced</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -79,8 +107,14 @@
       <alignment horizontal="general" vertical="top"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -400,10 +434,36 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{D0FF03EC-7A9B-4E50-ABEC-4AE7EE9B7A1D}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{0121CA9E-301C-40EF-A467-7BC7D02E2119}" mc:Ignorable="x14ac xr xr2 xr3">
   <dimension ref="A1:T200"/>
   <sheetFormatPr defaultRowHeight="15" defaultColWidth="8.8515625" customHeight="1"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" ht="15" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="A4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="1" orientation="portrait"/>

</xml_diff>